<commit_message>
Add Remote PC Bridge project media
Added the Remote PC Bridge portfolio entry and supporting media assets (video, poster, icon), plus generated content and manifest updates. The media generator was also hardened to validate generated video outputs and cache file hashes before reuse, preventing stale or invalid previews from being served.
</commit_message>
<xml_diff>
--- a/src/data/content/portfolio-master.xlsx
+++ b/src/data/content/portfolio-master.xlsx
@@ -9989,28 +9989,84 @@
       </c>
     </row>
     <row r="29" spans="1:4" ht="14.4" x14ac:dyDescent="0.3">
-      <c r="A29" s="16"/>
-      <c r="B29" s="16"/>
-      <c r="C29" s="16"/>
-      <c r="D29" s="22"/>
+      <c r="A29" s="16" t="inlineStr">
+        <is>
+          <t>6</t>
+        </is>
+      </c>
+      <c r="B29" s="16" t="inlineStr">
+        <is>
+          <t>C# / .NET 8</t>
+        </is>
+      </c>
+      <c r="C29" s="16">
+        <v>1</v>
+      </c>
+      <c r="D29" s="22" t="inlineStr">
+        <is>
+          <t>READY</t>
+        </is>
+      </c>
     </row>
     <row r="30" spans="1:4" ht="14.4" x14ac:dyDescent="0.3">
-      <c r="A30" s="20"/>
-      <c r="B30" s="20"/>
-      <c r="C30" s="20"/>
-      <c r="D30" s="22"/>
+      <c r="A30" s="20" t="inlineStr">
+        <is>
+          <t>6</t>
+        </is>
+      </c>
+      <c r="B30" s="20" t="inlineStr">
+        <is>
+          <t>ESP32 / Arduino</t>
+        </is>
+      </c>
+      <c r="C30" s="20">
+        <v>2</v>
+      </c>
+      <c r="D30" s="22" t="inlineStr">
+        <is>
+          <t>READY</t>
+        </is>
+      </c>
     </row>
     <row r="31" spans="1:4" ht="14.4" x14ac:dyDescent="0.3">
-      <c r="A31" s="16"/>
-      <c r="B31" s="16"/>
-      <c r="C31" s="16"/>
-      <c r="D31" s="22"/>
+      <c r="A31" s="16" t="inlineStr">
+        <is>
+          <t>6</t>
+        </is>
+      </c>
+      <c r="B31" s="16" t="inlineStr">
+        <is>
+          <t>Firebase Realtime Database</t>
+        </is>
+      </c>
+      <c r="C31" s="16">
+        <v>3</v>
+      </c>
+      <c r="D31" s="22" t="inlineStr">
+        <is>
+          <t>READY</t>
+        </is>
+      </c>
     </row>
     <row r="32" spans="1:4" ht="14.4" x14ac:dyDescent="0.3">
-      <c r="A32" s="20"/>
-      <c r="B32" s="20"/>
-      <c r="C32" s="20"/>
-      <c r="D32" s="22"/>
+      <c r="A32" s="20" t="inlineStr">
+        <is>
+          <t>6</t>
+        </is>
+      </c>
+      <c r="B32" s="20" t="inlineStr">
+        <is>
+          <t>Tailscale + Moonlight</t>
+        </is>
+      </c>
+      <c r="C32" s="20">
+        <v>4</v>
+      </c>
+      <c r="D32" s="22" t="inlineStr">
+        <is>
+          <t>READY</t>
+        </is>
+      </c>
     </row>
     <row r="33" spans="1:4" ht="14.4" x14ac:dyDescent="0.3">
       <c r="A33" s="16"/>
@@ -10512,28 +10568,84 @@
       </c>
     </row>
     <row r="29" spans="1:4" ht="14.4" x14ac:dyDescent="0.3">
-      <c r="A29" s="16"/>
-      <c r="B29" s="16"/>
-      <c r="C29" s="16"/>
-      <c r="D29" s="22"/>
+      <c r="A29" s="16" t="inlineStr">
+        <is>
+          <t>6</t>
+        </is>
+      </c>
+      <c r="B29" s="16" t="inlineStr">
+        <is>
+          <t>Windows Controller</t>
+        </is>
+      </c>
+      <c r="C29" s="16">
+        <v>1</v>
+      </c>
+      <c r="D29" s="22" t="inlineStr">
+        <is>
+          <t>READY</t>
+        </is>
+      </c>
     </row>
     <row r="30" spans="1:4" ht="14.4" x14ac:dyDescent="0.3">
-      <c r="A30" s="20"/>
-      <c r="B30" s="20"/>
-      <c r="C30" s="20"/>
-      <c r="D30" s="22"/>
+      <c r="A30" s="20" t="inlineStr">
+        <is>
+          <t>6</t>
+        </is>
+      </c>
+      <c r="B30" s="20" t="inlineStr">
+        <is>
+          <t>Firebase Command Bus</t>
+        </is>
+      </c>
+      <c r="C30" s="20">
+        <v>2</v>
+      </c>
+      <c r="D30" s="22" t="inlineStr">
+        <is>
+          <t>READY</t>
+        </is>
+      </c>
     </row>
     <row r="31" spans="1:4" ht="14.4" x14ac:dyDescent="0.3">
-      <c r="A31" s="16"/>
-      <c r="B31" s="16"/>
-      <c r="C31" s="16"/>
-      <c r="D31" s="22"/>
+      <c r="A31" s="16" t="inlineStr">
+        <is>
+          <t>6</t>
+        </is>
+      </c>
+      <c r="B31" s="16" t="inlineStr">
+        <is>
+          <t>ESP32 Wake-on-LAN</t>
+        </is>
+      </c>
+      <c r="C31" s="16">
+        <v>3</v>
+      </c>
+      <c r="D31" s="22" t="inlineStr">
+        <is>
+          <t>READY</t>
+        </is>
+      </c>
     </row>
     <row r="32" spans="1:4" ht="14.4" x14ac:dyDescent="0.3">
-      <c r="A32" s="20"/>
-      <c r="B32" s="20"/>
-      <c r="C32" s="20"/>
-      <c r="D32" s="22"/>
+      <c r="A32" s="20" t="inlineStr">
+        <is>
+          <t>6</t>
+        </is>
+      </c>
+      <c r="B32" s="20" t="inlineStr">
+        <is>
+          <t>Sunshine + Moonlight</t>
+        </is>
+      </c>
+      <c r="C32" s="20">
+        <v>4</v>
+      </c>
+      <c r="D32" s="22" t="inlineStr">
+        <is>
+          <t>READY</t>
+        </is>
+      </c>
     </row>
     <row r="33" spans="1:4" ht="14.4" x14ac:dyDescent="0.3">
       <c r="A33" s="16"/>
@@ -13387,21 +13499,75 @@
       </c>
     </row>
     <row r="14" spans="1:15" ht="14.4" x14ac:dyDescent="0.3">
-      <c r="A14" s="20"/>
-      <c r="B14" s="20"/>
-      <c r="C14" s="20"/>
-      <c r="D14" s="21"/>
-      <c r="E14" s="21"/>
-      <c r="F14" s="20"/>
-      <c r="G14" s="20"/>
-      <c r="H14" s="20"/>
-      <c r="I14" s="20"/>
-      <c r="J14" s="20"/>
-      <c r="K14" s="20"/>
-      <c r="L14" s="20"/>
-      <c r="M14" s="20"/>
-      <c r="N14" s="26"/>
-      <c r="O14" s="22"/>
+      <c r="A14" s="20">
+        <v>6</v>
+      </c>
+      <c r="B14" s="20" t="inlineStr">
+        <is>
+          <t>Remote PC Bridge</t>
+        </is>
+      </c>
+      <c r="C14" s="20" t="inlineStr">
+        <is>
+          <t>ESP32 Wake-on-LAN &amp; Remote Streaming Diagnostics</t>
+        </is>
+      </c>
+      <c r="D14" s="21" t="inlineStr">
+        <is>
+          <t>A home PC that is powered off cannot be reached through remote streaming, and failures across the wake and connection path are hard to pinpoint.</t>
+        </is>
+      </c>
+      <c r="E14" s="21" t="inlineStr">
+        <is>
+          <t>I built a Windows controller and ESP32 firmware that wake the PC over the home network, check each connection stage, and launch Moonlight when the desktop is ready.</t>
+        </is>
+      </c>
+      <c r="F14" s="20" t="inlineStr">
+        <is>
+          <t>https://github.com/Albjav12345/remote-pc-bridge</t>
+        </is>
+      </c>
+      <c r="G14" s="20" t="inlineStr">
+        <is>
+          <t>video</t>
+        </is>
+      </c>
+      <c r="H14" s="20" t="inlineStr">
+        <is>
+          <t>project-6-video</t>
+        </is>
+      </c>
+      <c r="I14" s="20" t="inlineStr">
+        <is>
+          <t>project-6-thumbnail</t>
+        </is>
+      </c>
+      <c r="J14" s="20" t="inlineStr">
+        <is>
+          <t>project-6-icon</t>
+        </is>
+      </c>
+      <c r="K14" s="20" t="inlineStr">
+        <is>
+          <t>auto</t>
+        </is>
+      </c>
+      <c r="L14" s="20">
+        <v>1</v>
+      </c>
+      <c r="M14" s="20">
+        <v>6</v>
+      </c>
+      <c r="N14" s="26" t="inlineStr">
+        <is>
+          <t>TRUE</t>
+        </is>
+      </c>
+      <c r="O14" s="22" t="inlineStr">
+        <is>
+          <t>READY</t>
+        </is>
+      </c>
     </row>
     <row r="15" spans="1:15" ht="14.4" x14ac:dyDescent="0.3">
       <c r="A15" s="16"/>
@@ -17729,14 +17895,46 @@
       </c>
     </row>
     <row r="45" spans="1:14" ht="14.4" x14ac:dyDescent="0.3">
-      <c r="A45" s="16"/>
-      <c r="B45" s="16"/>
-      <c r="C45" s="16"/>
-      <c r="D45" s="17"/>
-      <c r="E45" s="17"/>
-      <c r="F45" s="16"/>
-      <c r="G45" s="17"/>
-      <c r="H45" s="24"/>
+      <c r="A45" s="16" t="inlineStr">
+        <is>
+          <t>project-6-video</t>
+        </is>
+      </c>
+      <c r="B45" s="16" t="inlineStr">
+        <is>
+          <t>video</t>
+        </is>
+      </c>
+      <c r="C45" s="16" t="inlineStr">
+        <is>
+          <t>existing_public</t>
+        </is>
+      </c>
+      <c r="D45" s="17" t="inlineStr">
+        <is>
+          <t>/assets/projects/remote-pc-bridge.mp4</t>
+        </is>
+      </c>
+      <c r="E45" s="17" t="inlineStr">
+        <is>
+          <t>/assets/projects/remote-pc-bridge.mp4</t>
+        </is>
+      </c>
+      <c r="F45" s="16" t="inlineStr">
+        <is>
+          <t>Remote PC Bridge interface and PC demo</t>
+        </is>
+      </c>
+      <c r="G45" s="17" t="inlineStr">
+        <is>
+          <t>Master video from supplied project footage</t>
+        </is>
+      </c>
+      <c r="H45" s="24" t="inlineStr">
+        <is>
+          <t>TRUE</t>
+        </is>
+      </c>
       <c r="I45" s="28" t="str">
         <f t="shared" si="0"/>
         <v/>
@@ -17749,7 +17947,11 @@
         <f>IF($A45="","",IF(OR(UPPER($H45)&lt;&gt;"TRUE",$I45=""),"Unavailable",HYPERLINK("http://127.0.0.1:5173/__dev/asset-resolved"&amp;"?assetId="&amp;_xludf.ENCODEURL($A45)&amp;"&amp;sig="&amp;_xludf.ENCODEURL($B45&amp;"|"&amp;$C45&amp;"|"&amp;$D45&amp;"|"&amp;$E45&amp;"|"&amp;$H45),"Open resolved")))</f>
         <v/>
       </c>
-      <c r="L45" s="32"/>
+      <c r="L45" s="32" t="inlineStr">
+        <is>
+          <t>Remote PC Bridge video</t>
+        </is>
+      </c>
       <c r="M45" s="1" t="str">
         <f>IF($A45="","",HYPERLINK("#'ASSET_PREVIEW'!A45","Open preview"))</f>
         <v/>
@@ -17760,14 +17962,46 @@
       </c>
     </row>
     <row r="46" spans="1:14" ht="14.4" x14ac:dyDescent="0.3">
-      <c r="A46" s="20"/>
-      <c r="B46" s="20"/>
-      <c r="C46" s="20"/>
-      <c r="D46" s="21"/>
-      <c r="E46" s="21"/>
-      <c r="F46" s="20"/>
-      <c r="G46" s="21"/>
-      <c r="H46" s="26"/>
+      <c r="A46" s="20" t="inlineStr">
+        <is>
+          <t>project-6-thumbnail</t>
+        </is>
+      </c>
+      <c r="B46" s="20" t="inlineStr">
+        <is>
+          <t>image</t>
+        </is>
+      </c>
+      <c r="C46" s="20" t="inlineStr">
+        <is>
+          <t>existing_public</t>
+        </is>
+      </c>
+      <c r="D46" s="21" t="inlineStr">
+        <is>
+          <t>/assets/projects/remote-pc-bridge.jpg</t>
+        </is>
+      </c>
+      <c r="E46" s="21" t="inlineStr">
+        <is>
+          <t>/assets/projects/remote-pc-bridge.jpg</t>
+        </is>
+      </c>
+      <c r="F46" s="20" t="inlineStr">
+        <is>
+          <t>Remote PC Bridge dashboard in dark and light themes</t>
+        </is>
+      </c>
+      <c r="G46" s="21" t="inlineStr">
+        <is>
+          <t>Poster frame from supplied project footage</t>
+        </is>
+      </c>
+      <c r="H46" s="26" t="inlineStr">
+        <is>
+          <t>TRUE</t>
+        </is>
+      </c>
       <c r="I46" s="28" t="str">
         <f t="shared" si="0"/>
         <v/>
@@ -17780,7 +18014,11 @@
         <f>IF($A46="","",IF(OR(UPPER($H46)&lt;&gt;"TRUE",$I46=""),"Unavailable",HYPERLINK("http://127.0.0.1:5173/__dev/asset-resolved"&amp;"?assetId="&amp;_xludf.ENCODEURL($A46)&amp;"&amp;sig="&amp;_xludf.ENCODEURL($B46&amp;"|"&amp;$C46&amp;"|"&amp;$D46&amp;"|"&amp;$E46&amp;"|"&amp;$H46),"Open resolved")))</f>
         <v/>
       </c>
-      <c r="L46" s="32"/>
+      <c r="L46" s="32" t="inlineStr">
+        <is>
+          <t>Remote PC Bridge thumbnail</t>
+        </is>
+      </c>
       <c r="M46" s="1" t="str">
         <f>IF($A46="","",HYPERLINK("#'ASSET_PREVIEW'!A46","Open preview"))</f>
         <v/>
@@ -17791,14 +18029,46 @@
       </c>
     </row>
     <row r="47" spans="1:14" ht="14.4" x14ac:dyDescent="0.3">
-      <c r="A47" s="16"/>
-      <c r="B47" s="16"/>
-      <c r="C47" s="16"/>
-      <c r="D47" s="17"/>
-      <c r="E47" s="17"/>
-      <c r="F47" s="16"/>
-      <c r="G47" s="17"/>
-      <c r="H47" s="24"/>
+      <c r="A47" s="16" t="inlineStr">
+        <is>
+          <t>project-6-icon</t>
+        </is>
+      </c>
+      <c r="B47" s="16" t="inlineStr">
+        <is>
+          <t>icon</t>
+        </is>
+      </c>
+      <c r="C47" s="16" t="inlineStr">
+        <is>
+          <t>existing_public</t>
+        </is>
+      </c>
+      <c r="D47" s="17" t="inlineStr">
+        <is>
+          <t>/assets/projects/remote-pc-bridge-icon.png</t>
+        </is>
+      </c>
+      <c r="E47" s="17" t="inlineStr">
+        <is>
+          <t>/assets/projects/remote-pc-bridge-icon.png</t>
+        </is>
+      </c>
+      <c r="F47" s="16" t="inlineStr">
+        <is>
+          <t>Remote PC Bridge icon</t>
+        </is>
+      </c>
+      <c r="G47" s="17" t="inlineStr">
+        <is>
+          <t>Project icon</t>
+        </is>
+      </c>
+      <c r="H47" s="24" t="inlineStr">
+        <is>
+          <t>TRUE</t>
+        </is>
+      </c>
       <c r="I47" s="28" t="str">
         <f t="shared" si="0"/>
         <v/>
@@ -17811,7 +18081,11 @@
         <f>IF($A47="","",IF(OR(UPPER($H47)&lt;&gt;"TRUE",$I47=""),"Unavailable",HYPERLINK("http://127.0.0.1:5173/__dev/asset-resolved"&amp;"?assetId="&amp;_xludf.ENCODEURL($A47)&amp;"&amp;sig="&amp;_xludf.ENCODEURL($B47&amp;"|"&amp;$C47&amp;"|"&amp;$D47&amp;"|"&amp;$E47&amp;"|"&amp;$H47),"Open resolved")))</f>
         <v/>
       </c>
-      <c r="L47" s="32"/>
+      <c r="L47" s="32" t="inlineStr">
+        <is>
+          <t>Remote PC Bridge icon</t>
+        </is>
+      </c>
       <c r="M47" s="1" t="str">
         <f>IF($A47="","",HYPERLINK("#'ASSET_PREVIEW'!A47","Open preview"))</f>
         <v/>

</xml_diff>